<commit_message>
Changing question header to "grading criteria"
</commit_message>
<xml_diff>
--- a/demoGradeSheet.xlsx
+++ b/demoGradeSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vickihurd/GitHub/Customizable-Ultrasound-Grading-Platform/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C19B74B-930B-894D-937B-C49FE3EA5564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C4BD30F-3D9A-B642-9386-49E6216A92AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-35540" yWindow="1760" windowWidth="30240" windowHeight="18900" xr2:uid="{86FFFCC5-FE45-A243-B5A9-B435FBA1444F}"/>
   </bookViews>
@@ -473,9 +473,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -485,11 +482,14 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -834,164 +834,164 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" s="1" customFormat="1" ht="23" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="12"/>
-      <c r="P1" s="13"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="23"/>
     </row>
     <row r="2" spans="1:16" s="1" customFormat="1" ht="23" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15"/>
-      <c r="M2" s="15"/>
-      <c r="N2" s="16"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="17"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="13"/>
+      <c r="P2" s="14"/>
     </row>
     <row r="3" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
-      <c r="O3" s="19"/>
-      <c r="P3" s="20"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
+      <c r="M3" s="16"/>
+      <c r="N3" s="16"/>
+      <c r="O3" s="16"/>
+      <c r="P3" s="17"/>
     </row>
     <row r="4" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
-      <c r="O4" s="19"/>
-      <c r="P4" s="20"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="16"/>
+      <c r="J4" s="16"/>
+      <c r="K4" s="16"/>
+      <c r="L4" s="16"/>
+      <c r="M4" s="16"/>
+      <c r="N4" s="16"/>
+      <c r="O4" s="16"/>
+      <c r="P4" s="17"/>
     </row>
     <row r="5" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="19"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="19"/>
-      <c r="M5" s="19"/>
-      <c r="N5" s="19"/>
-      <c r="O5" s="19"/>
-      <c r="P5" s="20"/>
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="16"/>
+      <c r="K5" s="16"/>
+      <c r="L5" s="16"/>
+      <c r="M5" s="16"/>
+      <c r="N5" s="16"/>
+      <c r="O5" s="16"/>
+      <c r="P5" s="17"/>
     </row>
     <row r="6" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="19"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="19"/>
-      <c r="M6" s="19"/>
-      <c r="N6" s="19"/>
-      <c r="O6" s="19"/>
-      <c r="P6" s="20"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="16"/>
+      <c r="N6" s="16"/>
+      <c r="O6" s="16"/>
+      <c r="P6" s="17"/>
     </row>
     <row r="7" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="19"/>
-      <c r="L7" s="19"/>
-      <c r="M7" s="19"/>
-      <c r="N7" s="19"/>
-      <c r="O7" s="19"/>
-      <c r="P7" s="20"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="16"/>
+      <c r="N7" s="16"/>
+      <c r="O7" s="16"/>
+      <c r="P7" s="17"/>
     </row>
     <row r="8" spans="1:16" s="1" customFormat="1" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="B8" s="22"/>
-      <c r="C8" s="22"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="22"/>
-      <c r="F8" s="22"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="22"/>
-      <c r="I8" s="22"/>
-      <c r="J8" s="22"/>
-      <c r="K8" s="22"/>
-      <c r="L8" s="22"/>
-      <c r="M8" s="22"/>
-      <c r="N8" s="22"/>
-      <c r="O8" s="22"/>
-      <c r="P8" s="23"/>
+      <c r="B8" s="19"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
+      <c r="K8" s="19"/>
+      <c r="L8" s="19"/>
+      <c r="M8" s="19"/>
+      <c r="N8" s="19"/>
+      <c r="O8" s="19"/>
+      <c r="P8" s="20"/>
     </row>
     <row r="9" spans="1:16" s="1" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>

</xml_diff>